<commit_message>
Synthesis v2.1: replace report + inventory in place; add Caffrey2 round-2 memo
</commit_message>
<xml_diff>
--- a/Synthesis/gsib-board_duties-combined_inventory.xlsx
+++ b/Synthesis/gsib-board_duties-combined_inventory.xlsx
@@ -654,14 +654,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Board Duties at Category I U.S. GSIBs — Two-Layer Inventory (v2.0)</t>
+          <t>Board Duties at Category I U.S. GSIBs — Two-Layer Inventory (v2.1)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Critique-responsive edition: legal-force &amp; supervisory-consequence dimensions, duplicate clusters, burden model, reform roadmap, and a verification table.</t>
+          <t>Critique-responsive edition, v2.1: integrates the Caffrey2 supervisory-expectations memo — adds Credit risk, Fiduciary (trust), Director-eligibility/attestation, and Personal-liability entries; sharpens model-risk, resolution-cadence, BSA, cyber-timeline, and reliance-accommodation rows; reconciles counts against ~70-75 annual board actions; and adds feasibility-tiered reforms. New rows are Caffrey2-sourced; verify against primary sources before reliance.</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>June 24, 2026 (v2.1)</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>55 — In-force binding obligations only (statute, regulation, enforceable guideline). Excludes rescinded/unimplemented and all guidance.</t>
+          <t>68 — In-force binding obligations only (statute, regulation, enforceable guideline). Excludes rescinded/unimplemented and all guidance. (v2.0: 55; +13 in v2.1.)</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>83 — In-force binding obligations + supervisory expectations that are themselves rule-backed (cross-listed regulations).</t>
+          <t>98 — In-force binding obligations + supervisory expectations that are themselves rule-backed (cross-listed regulations). (v2.0: 83; +15 in v2.1.)</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>197 — All in-force board duties across both layers (binding obligations + all current supervisory expectations).</t>
+          <t>214 — All in-force board duties across both layers (binding obligations + all current supervisory expectations). (v2.0: 197; +17 in v2.1.)</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>23 — Distinct functional clusters the duties collapse into (the unit most relevant to reform).</t>
+          <t>26 — Distinct functional clusters the duties collapse into (the unit most relevant to reform). (v2.0: 23; +3 in v2.1. Personal-liability is a separate, non-reform cluster.)</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T209"/>
+  <dimension ref="A1:T230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2040,7 +2040,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>ALL BOARD DUTIES — combined two-layer master (v2.0)</t>
+          <t>ALL BOARD DUTIES — combined two-layer master (v2.1)</t>
         </is>
       </c>
     </row>
@@ -22819,6 +22819,2064 @@
       <c r="T209" s="9" t="inlineStr">
         <is>
           <t>Parallels operational-resilience resource expectation (OPR-02).</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B210" s="8" t="inlineStr">
+        <is>
+          <t>CRD-01</t>
+        </is>
+      </c>
+      <c r="C210" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="D210" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="E210" s="9" t="inlineStr">
+        <is>
+          <t>Board must adopt and review at least annually a written real-estate-lending policy consistent with safe-and-sound standards and the interagency Real Estate Lending Standards.</t>
+        </is>
+      </c>
+      <c r="F210" s="9" t="inlineStr">
+        <is>
+          <t>Real Estate Lending Standards (FRB/FDIC/OCC); FDI Act §304</t>
+        </is>
+      </c>
+      <c r="G210" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR 208 subpart E / 12 CFR 365 / 12 CFR 34 subpart D</t>
+        </is>
+      </c>
+      <c r="H210" s="9" t="n"/>
+      <c r="I210" s="9" t="inlineStr">
+        <is>
+          <t>FRB/FDIC/OCC</t>
+        </is>
+      </c>
+      <c r="J210" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K210" s="9" t="inlineStr">
+        <is>
+          <t>Full board</t>
+        </is>
+      </c>
+      <c r="L210" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M210" s="9" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="N210" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O210" s="9" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="P210" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy (parallel agency appendices)</t>
+        </is>
+      </c>
+      <c r="Q210" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R210" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S210" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T210" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Same annual policy-approval duty codified in parallel by OCC, FDIC, FRB. | Reform: One interagency real-estate-lending standard; single board approval satisfies all three.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B211" s="8" t="inlineStr">
+        <is>
+          <t>CRD-02</t>
+        </is>
+      </c>
+      <c r="C211" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="D211" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="E211" s="9" t="inlineStr">
+        <is>
+          <t>Board oversight of the allowance for credit losses (ACL/CECL) framework and methodology, ensuring an appropriate, well-documented allowance.</t>
+        </is>
+      </c>
+      <c r="F211" s="9" t="inlineStr">
+        <is>
+          <t>Interagency Policy Statement on Allowances for Credit Losses; FDI Act §39; ASC 326</t>
+        </is>
+      </c>
+      <c r="G211" s="9" t="inlineStr">
+        <is>
+          <t>Interagency ACL policy statement; ASC 326</t>
+        </is>
+      </c>
+      <c r="H211" s="9" t="n"/>
+      <c r="I211" s="9" t="inlineStr">
+        <is>
+          <t>FRB/FDIC/OCC</t>
+        </is>
+      </c>
+      <c r="J211" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K211" s="9" t="inlineStr">
+        <is>
+          <t>Full board or designated committee</t>
+        </is>
+      </c>
+      <c r="L211" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M211" s="9" t="inlineStr">
+        <is>
+          <t>Regulation / guidance</t>
+        </is>
+      </c>
+      <c r="N211" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O211" s="9" t="inlineStr">
+        <is>
+          <t>Quarterly / periodic</t>
+        </is>
+      </c>
+      <c r="P211" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="Q211" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R211" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S211" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T211" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: ACL governance overlaps audit-committee financial-reporting oversight and OCC/FRB credit-review expectations. | Reform: Fold ACL oversight into the audit/risk-committee credit cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B212" s="8" t="inlineStr">
+        <is>
+          <t>CRD-03</t>
+        </is>
+      </c>
+      <c r="C212" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="D212" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="E212" s="9" t="inlineStr">
+        <is>
+          <t>Board ensures an independent credit-risk-review (loan review) function whose findings are reported to the board or a committee.</t>
+        </is>
+      </c>
+      <c r="F212" s="9" t="inlineStr">
+        <is>
+          <t>Interagency Guidance on Credit Risk Review Systems (2020); OCC Heightened Standards App. D</t>
+        </is>
+      </c>
+      <c r="G212" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 30 App. D (independent risk mgmt)</t>
+        </is>
+      </c>
+      <c r="H212" s="9" t="n"/>
+      <c r="I212" s="9" t="inlineStr">
+        <is>
+          <t>FRB/FDIC/OCC</t>
+        </is>
+      </c>
+      <c r="J212" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K212" s="9" t="inlineStr">
+        <is>
+          <t>Full board or risk committee</t>
+        </is>
+      </c>
+      <c r="L212" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M212" s="9" t="inlineStr">
+        <is>
+          <t>Regulation / guidance</t>
+        </is>
+      </c>
+      <c r="N212" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O212" s="9" t="inlineStr">
+        <is>
+          <t>Periodic</t>
+        </is>
+      </c>
+      <c r="P212" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="Q212" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R212" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S212" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T212" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Overlaps OCC App. D independent-risk-management and audit oversight. | Reform: Cover within risk-committee credit reporting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B213" s="8" t="inlineStr">
+        <is>
+          <t>CRD-04</t>
+        </is>
+      </c>
+      <c r="C213" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="D213" s="9" t="inlineStr">
+        <is>
+          <t>Insider / affiliate / related-party</t>
+        </is>
+      </c>
+      <c r="E213" s="9" t="inlineStr">
+        <is>
+          <t>Prior board approval (majority of the entire board, interested party abstaining) of extensions of credit to executive officers, directors, principal shareholders, and their related interests above regulatory thresholds.</t>
+        </is>
+      </c>
+      <c r="F213" s="9" t="inlineStr">
+        <is>
+          <t>Federal Reserve Act §22(h); Regulation O</t>
+        </is>
+      </c>
+      <c r="G213" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 215; 12 U.S.C. 375b(3)</t>
+        </is>
+      </c>
+      <c r="H213" s="9" t="n"/>
+      <c r="I213" s="9" t="inlineStr">
+        <is>
+          <t>FRB</t>
+        </is>
+      </c>
+      <c r="J213" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K213" s="9" t="inlineStr">
+        <is>
+          <t>Majority of the entire board</t>
+        </is>
+      </c>
+      <c r="L213" s="9" t="inlineStr">
+        <is>
+          <t>Each insider (abstention)</t>
+        </is>
+      </c>
+      <c r="M213" s="9" t="inlineStr">
+        <is>
+          <t>Statute / Regulation</t>
+        </is>
+      </c>
+      <c r="N213" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O213" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven</t>
+        </is>
+      </c>
+      <c r="P213" s="10" t="inlineStr">
+        <is>
+          <t>Limited overlap (distinct insured-bank protection)</t>
+        </is>
+      </c>
+      <c r="Q213" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R213" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S213" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T213" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Specific board-approval trigger within the Reg O regime catalogued at a higher level in domain 11. | Reform: Retain; protects the insured bank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B214" s="8" t="inlineStr">
+        <is>
+          <t>CRD-05</t>
+        </is>
+      </c>
+      <c r="C214" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="D214" s="9" t="inlineStr">
+        <is>
+          <t>Insider / affiliate / related-party</t>
+        </is>
+      </c>
+      <c r="E214" s="9" t="inlineStr">
+        <is>
+          <t>Discrete affiliate-transaction board approvals under Regulation W: affiliate-underwritten securities purchases (§223.53(b)), affiliate loan-participation renewals (§223.15(b)(2)), and internal-reorganization asset purchases exempted from §23A (§223.41(d)).</t>
+        </is>
+      </c>
+      <c r="F214" s="9" t="inlineStr">
+        <is>
+          <t>Regulation W; Federal Reserve Act §23A/§23B</t>
+        </is>
+      </c>
+      <c r="G214" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 223; 12 U.S.C. 371c-1</t>
+        </is>
+      </c>
+      <c r="H214" s="9" t="n"/>
+      <c r="I214" s="9" t="inlineStr">
+        <is>
+          <t>FRB</t>
+        </is>
+      </c>
+      <c r="J214" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K214" s="9" t="inlineStr">
+        <is>
+          <t>Majority of the board</t>
+        </is>
+      </c>
+      <c r="L214" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M214" s="9" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="N214" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O214" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven</t>
+        </is>
+      </c>
+      <c r="P214" s="10" t="inlineStr">
+        <is>
+          <t>Limited overlap (parallel-but-justified)</t>
+        </is>
+      </c>
+      <c r="Q214" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R214" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S214" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T214" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Granular board-approval triggers within the Reg W framework. | Reform: Where permitted, approve standards subject to periodic review rather than transaction-by-transaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B215" s="8" t="inlineStr">
+        <is>
+          <t>CRD-06</t>
+        </is>
+      </c>
+      <c r="C215" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="D215" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="E215" s="9" t="inlineStr">
+        <is>
+          <t>Board oversight of correspondent credit-concentration policies limiting exposure to individual correspondent banks.</t>
+        </is>
+      </c>
+      <c r="F215" s="9" t="inlineStr">
+        <is>
+          <t>Regulation F</t>
+        </is>
+      </c>
+      <c r="G215" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 206</t>
+        </is>
+      </c>
+      <c r="H215" s="9" t="n"/>
+      <c r="I215" s="9" t="inlineStr">
+        <is>
+          <t>FRB</t>
+        </is>
+      </c>
+      <c r="J215" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K215" s="9" t="inlineStr">
+        <is>
+          <t>Full board or designated committee</t>
+        </is>
+      </c>
+      <c r="L215" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M215" s="9" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="N215" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O215" s="9" t="inlineStr">
+        <is>
+          <t>Periodic</t>
+        </is>
+      </c>
+      <c r="P215" s="10" t="inlineStr">
+        <is>
+          <t>Unique / limited overlap</t>
+        </is>
+      </c>
+      <c r="Q215" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R215" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S215" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T215" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Folds into enterprise credit-concentration and counterparty-limit monitoring. | Reform: Cover within risk-committee limit monitoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B216" s="8" t="inlineStr">
+        <is>
+          <t>FID-01</t>
+        </is>
+      </c>
+      <c r="C216" s="9" t="inlineStr">
+        <is>
+          <t>Fiduciary (trust) governance</t>
+        </is>
+      </c>
+      <c r="D216" s="9" t="inlineStr">
+        <is>
+          <t>Fiduciary (trust) governance</t>
+        </is>
+      </c>
+      <c r="E216" s="9" t="inlineStr">
+        <is>
+          <t>The bank's fiduciary activities must be managed by or under the direction of its board, and the board must adopt written policies governing fiduciary activities.</t>
+        </is>
+      </c>
+      <c r="F216" s="9" t="inlineStr">
+        <is>
+          <t>OCC fiduciary-activities rule (national banks); FSA counterpart</t>
+        </is>
+      </c>
+      <c r="G216" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR 9.4(a); 12 CFR 9.5; 12 CFR part 150</t>
+        </is>
+      </c>
+      <c r="H216" s="9" t="n"/>
+      <c r="I216" s="9" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="J216" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K216" s="9" t="inlineStr">
+        <is>
+          <t>Full board</t>
+        </is>
+      </c>
+      <c r="L216" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M216" s="9" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="N216" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O216" s="9" t="inlineStr">
+        <is>
+          <t>Periodic / annual</t>
+        </is>
+      </c>
+      <c r="P216" s="10" t="inlineStr">
+        <is>
+          <t>Unique / limited overlap</t>
+        </is>
+      </c>
+      <c r="Q216" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R216" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S216" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T216" s="9" t="inlineStr">
+        <is>
+          <t>Most material to custody/trust GSIBs (BNY, State Street). | Overlap: Distinct from enterprise risk governance; trust-charter-specific. | Reform: Retain; distinct statutory purpose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B217" s="8" t="inlineStr">
+        <is>
+          <t>FID-02</t>
+        </is>
+      </c>
+      <c r="C217" s="9" t="inlineStr">
+        <is>
+          <t>Fiduciary (trust) governance</t>
+        </is>
+      </c>
+      <c r="D217" s="9" t="inlineStr">
+        <is>
+          <t>Audit committee &amp; independence</t>
+        </is>
+      </c>
+      <c r="E217" s="9" t="inlineStr">
+        <is>
+          <t>A fiduciary audit committee of directors (excluding officers significantly involved in fiduciary administration) must arrange suitable audits of fiduciary activities at least annually.</t>
+        </is>
+      </c>
+      <c r="F217" s="9" t="inlineStr">
+        <is>
+          <t>OCC fiduciary-activities rule</t>
+        </is>
+      </c>
+      <c r="G217" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR 9.9</t>
+        </is>
+      </c>
+      <c r="H217" s="9" t="n"/>
+      <c r="I217" s="9" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="J217" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K217" s="9" t="inlineStr">
+        <is>
+          <t>Fiduciary audit committee</t>
+        </is>
+      </c>
+      <c r="L217" s="9" t="inlineStr">
+        <is>
+          <t>Excludes officers in fiduciary admin</t>
+        </is>
+      </c>
+      <c r="M217" s="9" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="N217" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP); rating downgrade</t>
+        </is>
+      </c>
+      <c r="O217" s="9" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="P217" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="Q217" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R217" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S217" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T217" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Parallels the §36 / Part 363 audit committee but covers fiduciary activities specifically. | Reform: Permit the §36 audit committee to satisfy the fiduciary-audit duty where composition overlaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B218" s="8" t="inlineStr">
+        <is>
+          <t>FID-03</t>
+        </is>
+      </c>
+      <c r="C218" s="9" t="inlineStr">
+        <is>
+          <t>Fiduciary (trust) governance</t>
+        </is>
+      </c>
+      <c r="D218" s="9" t="inlineStr">
+        <is>
+          <t>Fiduciary (trust) governance</t>
+        </is>
+      </c>
+      <c r="E218" s="9" t="inlineStr">
+        <is>
+          <t>Collective investment funds must operate under a board-approved written plan; fiduciary assets must be held in the joint custody of at least two designated officers.</t>
+        </is>
+      </c>
+      <c r="F218" s="9" t="inlineStr">
+        <is>
+          <t>OCC fiduciary-activities rule</t>
+        </is>
+      </c>
+      <c r="G218" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR 9.18(b)(1); 12 CFR 9.13(a)</t>
+        </is>
+      </c>
+      <c r="H218" s="9" t="n"/>
+      <c r="I218" s="9" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="J218" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K218" s="9" t="inlineStr">
+        <is>
+          <t>Full board</t>
+        </is>
+      </c>
+      <c r="L218" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M218" s="9" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="N218" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement (cease-and-desist, CMP)</t>
+        </is>
+      </c>
+      <c r="O218" s="9" t="inlineStr">
+        <is>
+          <t>Periodic</t>
+        </is>
+      </c>
+      <c r="P218" s="10" t="inlineStr">
+        <is>
+          <t>Unique / limited overlap</t>
+        </is>
+      </c>
+      <c r="Q218" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R218" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S218" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T218" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Operational fiduciary control; minimal cross-regulator overlap. | Reform: Retain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B219" s="8" t="inlineStr">
+        <is>
+          <t>ELG-01</t>
+        </is>
+      </c>
+      <c r="C219" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility, attestation &amp; continuity</t>
+        </is>
+      </c>
+      <c r="D219" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility &amp; continuity</t>
+        </is>
+      </c>
+      <c r="E219" s="9" t="inlineStr">
+        <is>
+          <t>A bank in troubled condition or not meeting minimum capital must give the agency 30 days' written notice before adding or replacing a director or senior executive officer (the '914 process'), with CBCA/FFIEC background information; a disapproved individual may not serve while an appeal is pending.</t>
+        </is>
+      </c>
+      <c r="F219" s="9" t="inlineStr">
+        <is>
+          <t>Change in director/SEO statute; FRB Reg Y; OCC rule</t>
+        </is>
+      </c>
+      <c r="G219" s="9" t="inlineStr">
+        <is>
+          <t>12 U.S.C. 1831i; 12 CFR 225.71-.73; 12 CFR 5.51</t>
+        </is>
+      </c>
+      <c r="H219" s="9" t="n"/>
+      <c r="I219" s="9" t="inlineStr">
+        <is>
+          <t>FRB/OCC</t>
+        </is>
+      </c>
+      <c r="J219" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K219" s="9" t="inlineStr">
+        <is>
+          <t>Full board / institution</t>
+        </is>
+      </c>
+      <c r="L219" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M219" s="9" t="inlineStr">
+        <is>
+          <t>Statute / Regulation</t>
+        </is>
+      </c>
+      <c r="N219" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement; disapproval bars service</t>
+        </is>
+      </c>
+      <c r="O219" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven</t>
+        </is>
+      </c>
+      <c r="P219" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy (parallel FRB/OCC processes)</t>
+        </is>
+      </c>
+      <c r="Q219" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R219" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S219" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T219" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Parallel FRB and OCC change-in-director notice regimes. | Reform: Single interagency change-in-director notice procedure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B220" s="8" t="inlineStr">
+        <is>
+          <t>ELG-02</t>
+        </is>
+      </c>
+      <c r="C220" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility, attestation &amp; continuity</t>
+        </is>
+      </c>
+      <c r="D220" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility &amp; continuity</t>
+        </is>
+      </c>
+      <c r="E220" s="9" t="inlineStr">
+        <is>
+          <t>Statutory disqualification: a person convicted of (or in pretrial diversion for) a crime involving dishonesty, breach of trust, or money laundering is barred from serving as an institution-affiliated party absent agency consent; a removal/prohibition order terminates the directorship on service.</t>
+        </is>
+      </c>
+      <c r="F220" s="9" t="inlineStr">
+        <is>
+          <t>Crime/IAP disqualification statute; FDIA removal authorities</t>
+        </is>
+      </c>
+      <c r="G220" s="9" t="inlineStr">
+        <is>
+          <t>12 U.S.C. 1829; FDI Act §8(e), §8(g)</t>
+        </is>
+      </c>
+      <c r="H220" s="9" t="n"/>
+      <c r="I220" s="9" t="inlineStr">
+        <is>
+          <t>Banking agencies</t>
+        </is>
+      </c>
+      <c r="J220" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K220" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="L220" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="M220" s="9" t="inlineStr">
+        <is>
+          <t>Statute</t>
+        </is>
+      </c>
+      <c r="N220" s="9" t="inlineStr">
+        <is>
+          <t>Automatic bar; criminal/CMP exposure</t>
+        </is>
+      </c>
+      <c r="O220" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven</t>
+        </is>
+      </c>
+      <c r="P220" s="10" t="inlineStr">
+        <is>
+          <t>Unique / limited overlap</t>
+        </is>
+      </c>
+      <c r="Q220" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R220" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S220" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T220" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Director-level eligibility bar. | Reform: Retain; statutory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B221" s="8" t="inlineStr">
+        <is>
+          <t>ELG-03</t>
+        </is>
+      </c>
+      <c r="C221" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility, attestation &amp; continuity</t>
+        </is>
+      </c>
+      <c r="D221" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility &amp; continuity</t>
+        </is>
+      </c>
+      <c r="E221" s="9" t="inlineStr">
+        <is>
+          <t>The correctness of each Call Report (report of condition) must be attested by at least two directors (three for a national bank) other than the declaring officer; directors review and sign the report of examination; a change of CEO or director is reported promptly on a change in control.</t>
+        </is>
+      </c>
+      <c r="F221" s="9" t="inlineStr">
+        <is>
+          <t>FDI Act §7(a)(3); FDI Act §7(j); OCC Comptroller's Licensing Manual</t>
+        </is>
+      </c>
+      <c r="G221" s="9" t="inlineStr">
+        <is>
+          <t>FDI Act §7(a)(3); §7(j)</t>
+        </is>
+      </c>
+      <c r="H221" s="9" t="n"/>
+      <c r="I221" s="9" t="inlineStr">
+        <is>
+          <t>FDIC/OCC</t>
+        </is>
+      </c>
+      <c r="J221" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K221" s="9" t="inlineStr">
+        <is>
+          <t>Designated directors</t>
+        </is>
+      </c>
+      <c r="L221" s="9" t="inlineStr">
+        <is>
+          <t>Two/three directors</t>
+        </is>
+      </c>
+      <c r="M221" s="9" t="inlineStr">
+        <is>
+          <t>Statute / Regulation</t>
+        </is>
+      </c>
+      <c r="N221" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement; false-entry exposure</t>
+        </is>
+      </c>
+      <c r="O221" s="9" t="inlineStr">
+        <is>
+          <t>Quarterly / event-driven</t>
+        </is>
+      </c>
+      <c r="P221" s="10" t="inlineStr">
+        <is>
+          <t>Unique / limited overlap</t>
+        </is>
+      </c>
+      <c r="Q221" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R221" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S221" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T221" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Recurring attestation duty; low marginal burden. | Reform: Retain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="7" t="inlineStr">
+        <is>
+          <t>Binding obligation</t>
+        </is>
+      </c>
+      <c r="B222" s="8" t="inlineStr">
+        <is>
+          <t>ELG-04</t>
+        </is>
+      </c>
+      <c r="C222" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility, attestation &amp; continuity</t>
+        </is>
+      </c>
+      <c r="D222" s="9" t="inlineStr">
+        <is>
+          <t>Incentive compensation</t>
+        </is>
+      </c>
+      <c r="E222" s="9" t="inlineStr">
+        <is>
+          <t>Board determinations governing indemnification of institution-affiliated parties (good-faith / best-interests / no-material-adverse-safety-and-soundness findings, with interested-party recusal) and golden-parachute and severance payments under the Part 359 prohibitions and permitted-payment exceptions.</t>
+        </is>
+      </c>
+      <c r="F222" s="9" t="inlineStr">
+        <is>
+          <t>FDIC golden-parachute &amp; indemnification rule; FDI Act §18(k)</t>
+        </is>
+      </c>
+      <c r="G222" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 359; FDI Act §18(k)</t>
+        </is>
+      </c>
+      <c r="H222" s="9" t="n"/>
+      <c r="I222" s="9" t="inlineStr">
+        <is>
+          <t>FDIC</t>
+        </is>
+      </c>
+      <c r="J222" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K222" s="9" t="inlineStr">
+        <is>
+          <t>Full board</t>
+        </is>
+      </c>
+      <c r="L222" s="9" t="inlineStr">
+        <is>
+          <t>Interested-party recusal</t>
+        </is>
+      </c>
+      <c r="M222" s="9" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="N222" s="9" t="inlineStr">
+        <is>
+          <t>Enforcement; prohibited-payment liability</t>
+        </is>
+      </c>
+      <c r="O222" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven</t>
+        </is>
+      </c>
+      <c r="P222" s="10" t="inlineStr">
+        <is>
+          <t>Limited overlap (distinct DIF protection)</t>
+        </is>
+      </c>
+      <c r="Q222" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R222" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S222" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T222" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Distinct from incentive-compensation governance; protects the insured bank and the Deposit Insurance Fund. | Reform: Retain; coordinate with a finalized §956 framework if adopted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="14" t="inlineStr">
+        <is>
+          <t>Supervisory expectation</t>
+        </is>
+      </c>
+      <c r="B223" s="8" t="inlineStr">
+        <is>
+          <t>CRX-01</t>
+        </is>
+      </c>
+      <c r="C223" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk oversight (supervisory)</t>
+        </is>
+      </c>
+      <c r="D223" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="E223" s="9" t="inlineStr">
+        <is>
+          <t>Board oversight of credit-risk appetite, concentration limits, and credit-administration quality; review of problem-asset and ACL trends through periodic MIS.</t>
+        </is>
+      </c>
+      <c r="F223" s="9" t="inlineStr">
+        <is>
+          <t>OCC Comptroller's Handbook (Concentrations of Credit; Allowances); Fed Commercial Bank Examination Manual; credit-risk SR letters</t>
+        </is>
+      </c>
+      <c r="G223" s="9" t="inlineStr">
+        <is>
+          <t>Credit-risk handbook/manual sections</t>
+        </is>
+      </c>
+      <c r="H223" s="9" t="n"/>
+      <c r="I223" s="9" t="inlineStr">
+        <is>
+          <t>OCC/FRB</t>
+        </is>
+      </c>
+      <c r="J223" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K223" s="9" t="inlineStr">
+        <is>
+          <t>Full board or risk/credit committee</t>
+        </is>
+      </c>
+      <c r="L223" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M223" s="9" t="inlineStr">
+        <is>
+          <t>Supervisory guidance</t>
+        </is>
+      </c>
+      <c r="N223" s="9" t="inlineStr">
+        <is>
+          <t>Exam findings / MRAs; informs ratings (no direct legal force)</t>
+        </is>
+      </c>
+      <c r="O223" s="9" t="inlineStr">
+        <is>
+          <t>Periodic</t>
+        </is>
+      </c>
+      <c r="P223" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="Q223" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R223" s="9" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S223" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T223" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Elaborates the binding real-estate-lending and ACL duties. | Reform: Cross-reference the handbook to the rule; avoid restating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="14" t="inlineStr">
+        <is>
+          <t>Supervisory expectation</t>
+        </is>
+      </c>
+      <c r="B224" s="8" t="inlineStr">
+        <is>
+          <t>CRX-02</t>
+        </is>
+      </c>
+      <c r="C224" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk oversight (supervisory)</t>
+        </is>
+      </c>
+      <c r="D224" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="E224" s="9" t="inlineStr">
+        <is>
+          <t>Board or committee oversight of counterparty credit risk and, where applicable, leveraged-lending risk-appetite and exception reporting.</t>
+        </is>
+      </c>
+      <c r="F224" s="9" t="inlineStr">
+        <is>
+          <t>SR 11-10 / interagency counterparty guidance; 2013 Interagency Leveraged Lending Guidance (enforcement-deprioritized)</t>
+        </is>
+      </c>
+      <c r="G224" s="9" t="inlineStr">
+        <is>
+          <t>SR 11-10; 2013 leveraged-lending guidance</t>
+        </is>
+      </c>
+      <c r="H224" s="9" t="n"/>
+      <c r="I224" s="9" t="inlineStr">
+        <is>
+          <t>FRB/OCC/FDIC</t>
+        </is>
+      </c>
+      <c r="J224" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K224" s="9" t="inlineStr">
+        <is>
+          <t>Risk / credit committee</t>
+        </is>
+      </c>
+      <c r="L224" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M224" s="9" t="inlineStr">
+        <is>
+          <t>Supervisory guidance</t>
+        </is>
+      </c>
+      <c r="N224" s="9" t="inlineStr">
+        <is>
+          <t>Exam findings / MRAs; informs ratings (no direct legal force)</t>
+        </is>
+      </c>
+      <c r="O224" s="9" t="inlineStr">
+        <is>
+          <t>Periodic</t>
+        </is>
+      </c>
+      <c r="P224" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="Q224" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R224" s="9" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S224" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T224" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Overlaps enterprise risk-limit monitoring. | Reform: Fold into risk-committee limit oversight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="14" t="inlineStr">
+        <is>
+          <t>Supervisory expectation</t>
+        </is>
+      </c>
+      <c r="B225" s="8" t="inlineStr">
+        <is>
+          <t>CCX-01</t>
+        </is>
+      </c>
+      <c r="C225" s="9" t="inlineStr">
+        <is>
+          <t>Additional consumer &amp; compliance oversight</t>
+        </is>
+      </c>
+      <c r="D225" s="9" t="inlineStr">
+        <is>
+          <t>Consumer compliance (CMS)</t>
+        </is>
+      </c>
+      <c r="E225" s="9" t="inlineStr">
+        <is>
+          <t>Board oversight that strategic plans consider community credit needs and CRA performance.</t>
+        </is>
+      </c>
+      <c r="F225" s="9" t="inlineStr">
+        <is>
+          <t>Community Reinvestment Act; OCC Director's Reference Guide</t>
+        </is>
+      </c>
+      <c r="G225" s="9" t="inlineStr">
+        <is>
+          <t>12 U.S.C. 2901 et seq.</t>
+        </is>
+      </c>
+      <c r="H225" s="9" t="n"/>
+      <c r="I225" s="9" t="inlineStr">
+        <is>
+          <t>OCC/FRB/FDIC</t>
+        </is>
+      </c>
+      <c r="J225" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K225" s="9" t="inlineStr">
+        <is>
+          <t>Full board</t>
+        </is>
+      </c>
+      <c r="L225" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M225" s="9" t="inlineStr">
+        <is>
+          <t>Statute / supervisory guidance</t>
+        </is>
+      </c>
+      <c r="N225" s="9" t="inlineStr">
+        <is>
+          <t>Exam findings; CRA rating</t>
+        </is>
+      </c>
+      <c r="O225" s="9" t="inlineStr">
+        <is>
+          <t>Periodic</t>
+        </is>
+      </c>
+      <c r="P225" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="Q225" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R225" s="9" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S225" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T225" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Distinct consumer mandate. | Reform: Coordinate within the CMS oversight cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="14" t="inlineStr">
+        <is>
+          <t>Supervisory expectation</t>
+        </is>
+      </c>
+      <c r="B226" s="8" t="inlineStr">
+        <is>
+          <t>CCX-02</t>
+        </is>
+      </c>
+      <c r="C226" s="9" t="inlineStr">
+        <is>
+          <t>Additional consumer &amp; compliance oversight</t>
+        </is>
+      </c>
+      <c r="D226" s="9" t="inlineStr">
+        <is>
+          <t>Consumer compliance (CMS)</t>
+        </is>
+      </c>
+      <c r="E226" s="9" t="inlineStr">
+        <is>
+          <t>Board oversight of compliance with the FDIC deposit-insurance representation/advertising rules (Part 328) and, for FX-active firms, oversight of the foreign-exchange-settlement compliance function.</t>
+        </is>
+      </c>
+      <c r="F226" s="9" t="inlineStr">
+        <is>
+          <t>FDIC deposit-insurance representation rule; SR 13-24</t>
+        </is>
+      </c>
+      <c r="G226" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 328; SR 13-24</t>
+        </is>
+      </c>
+      <c r="H226" s="9" t="n"/>
+      <c r="I226" s="9" t="inlineStr">
+        <is>
+          <t>FDIC/FRB</t>
+        </is>
+      </c>
+      <c r="J226" s="9" t="inlineStr">
+        <is>
+          <t>IDI</t>
+        </is>
+      </c>
+      <c r="K226" s="9" t="inlineStr">
+        <is>
+          <t>Full board or committee</t>
+        </is>
+      </c>
+      <c r="L226" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M226" s="9" t="inlineStr">
+        <is>
+          <t>Regulation / supervisory guidance</t>
+        </is>
+      </c>
+      <c r="N226" s="9" t="inlineStr">
+        <is>
+          <t>Exam findings / MRAs</t>
+        </is>
+      </c>
+      <c r="O226" s="9" t="inlineStr">
+        <is>
+          <t>Periodic</t>
+        </is>
+      </c>
+      <c r="P226" s="10" t="inlineStr">
+        <is>
+          <t>Unique / limited overlap</t>
+        </is>
+      </c>
+      <c r="Q226" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R226" s="9" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S226" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T226" s="9" t="inlineStr">
+        <is>
+          <t>Overlap: Discrete conduct items. | Reform: Coordinate within the CMS oversight cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="7" t="inlineStr">
+        <is>
+          <t>Personal liability (individual director)</t>
+        </is>
+      </c>
+      <c r="B227" s="8" t="inlineStr">
+        <is>
+          <t>PLB-01</t>
+        </is>
+      </c>
+      <c r="C227" s="9" t="inlineStr">
+        <is>
+          <t>Personal &amp; individual-director liability</t>
+        </is>
+      </c>
+      <c r="D227" s="9" t="inlineStr">
+        <is>
+          <t>Personal liability</t>
+        </is>
+      </c>
+      <c r="E227" s="9" t="inlineStr">
+        <is>
+          <t>Criminal liability for false entries: every director of a bank or BHC is subject to the same criminal penalties for false entries.</t>
+        </is>
+      </c>
+      <c r="F227" s="9" t="inlineStr">
+        <is>
+          <t>False-entries criminal statute</t>
+        </is>
+      </c>
+      <c r="G227" s="9" t="inlineStr">
+        <is>
+          <t>18 U.S.C. 1005; 12 U.S.C. 1847(a)(2)</t>
+        </is>
+      </c>
+      <c r="H227" s="9" t="n"/>
+      <c r="I227" s="9" t="inlineStr">
+        <is>
+          <t>DOJ / banking agencies</t>
+        </is>
+      </c>
+      <c r="J227" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K227" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="L227" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="M227" s="9" t="inlineStr">
+        <is>
+          <t>Statute</t>
+        </is>
+      </c>
+      <c r="N227" s="9" t="inlineStr">
+        <is>
+          <t>Criminal</t>
+        </is>
+      </c>
+      <c r="O227" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven</t>
+        </is>
+      </c>
+      <c r="P227" s="10" t="inlineStr">
+        <is>
+          <t>n/a (individual)</t>
+        </is>
+      </c>
+      <c r="Q227" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R227" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S227" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T227" s="9" t="inlineStr">
+        <is>
+          <t>Analytically distinct: individual exposure, NOT counted as a recurring board action or in the burden model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="7" t="inlineStr">
+        <is>
+          <t>Personal liability (individual director)</t>
+        </is>
+      </c>
+      <c r="B228" s="8" t="inlineStr">
+        <is>
+          <t>PLB-02</t>
+        </is>
+      </c>
+      <c r="C228" s="9" t="inlineStr">
+        <is>
+          <t>Personal &amp; individual-director liability</t>
+        </is>
+      </c>
+      <c r="D228" s="9" t="inlineStr">
+        <is>
+          <t>Personal liability</t>
+        </is>
+      </c>
+      <c r="E228" s="9" t="inlineStr">
+        <is>
+          <t>Removal and prohibition: an institution-affiliated party may be removed/prohibited for misconduct, and a director with knowledge of a violation must take action to stop or prevent recurrence.</t>
+        </is>
+      </c>
+      <c r="F228" s="9" t="inlineStr">
+        <is>
+          <t>FDIA removal/prohibition authority</t>
+        </is>
+      </c>
+      <c r="G228" s="9" t="inlineStr">
+        <is>
+          <t>FDI Act §8(e); §8(e)(2)(B)</t>
+        </is>
+      </c>
+      <c r="H228" s="9" t="n"/>
+      <c r="I228" s="9" t="inlineStr">
+        <is>
+          <t>Banking agencies</t>
+        </is>
+      </c>
+      <c r="J228" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K228" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="L228" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="M228" s="9" t="inlineStr">
+        <is>
+          <t>Statute</t>
+        </is>
+      </c>
+      <c r="N228" s="9" t="inlineStr">
+        <is>
+          <t>Removal/prohibition; CMP</t>
+        </is>
+      </c>
+      <c r="O228" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven</t>
+        </is>
+      </c>
+      <c r="P228" s="10" t="inlineStr">
+        <is>
+          <t>n/a (individual)</t>
+        </is>
+      </c>
+      <c r="Q228" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R228" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S228" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T228" s="9" t="inlineStr">
+        <is>
+          <t>Analytically distinct: individual exposure; bears on the risk calculus of board service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="7" t="inlineStr">
+        <is>
+          <t>Personal liability (individual director)</t>
+        </is>
+      </c>
+      <c r="B229" s="8" t="inlineStr">
+        <is>
+          <t>PLB-03</t>
+        </is>
+      </c>
+      <c r="C229" s="9" t="inlineStr">
+        <is>
+          <t>Personal &amp; individual-director liability</t>
+        </is>
+      </c>
+      <c r="D229" s="9" t="inlineStr">
+        <is>
+          <t>Personal liability</t>
+        </is>
+      </c>
+      <c r="E229" s="9" t="inlineStr">
+        <is>
+          <t>Receivership / orderly-liquidation liability: personal liability for gross negligence in FDIC-as-receiver actions, and §210(s) compensation recoupment from directors 'substantially responsible' for the failure under a negligence standard, with the burden on the director.</t>
+        </is>
+      </c>
+      <c r="F229" s="9" t="inlineStr">
+        <is>
+          <t>FIRREA director-liability; Dodd-Frank Title II</t>
+        </is>
+      </c>
+      <c r="G229" s="9" t="inlineStr">
+        <is>
+          <t>12 U.S.C. 1821(k); 12 U.S.C. 5390(f); 12 U.S.C. 5390(s); 12 CFR 380.7</t>
+        </is>
+      </c>
+      <c r="H229" s="9" t="n"/>
+      <c r="I229" s="9" t="inlineStr">
+        <is>
+          <t>FDIC</t>
+        </is>
+      </c>
+      <c r="J229" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K229" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="L229" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="M229" s="9" t="inlineStr">
+        <is>
+          <t>Statute</t>
+        </is>
+      </c>
+      <c r="N229" s="9" t="inlineStr">
+        <is>
+          <t>Monetary damages; comp recoupment</t>
+        </is>
+      </c>
+      <c r="O229" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven (resolution)</t>
+        </is>
+      </c>
+      <c r="P229" s="10" t="inlineStr">
+        <is>
+          <t>n/a (individual)</t>
+        </is>
+      </c>
+      <c r="Q229" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R229" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S229" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T229" s="9" t="inlineStr">
+        <is>
+          <t>Two culpability standards — gross negligence for damages, simple negligence for recoupment. Analytically distinct; not a recurring board action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="7" t="inlineStr">
+        <is>
+          <t>Personal liability (individual director)</t>
+        </is>
+      </c>
+      <c r="B230" s="8" t="inlineStr">
+        <is>
+          <t>PLB-04</t>
+        </is>
+      </c>
+      <c r="C230" s="9" t="inlineStr">
+        <is>
+          <t>Personal &amp; individual-director liability</t>
+        </is>
+      </c>
+      <c r="D230" s="9" t="inlineStr">
+        <is>
+          <t>Personal liability</t>
+        </is>
+      </c>
+      <c r="E230" s="9" t="inlineStr">
+        <is>
+          <t>Indemnification limits, D&amp;O insurance, and fidelity bonds: Part 359 prohibits indemnifying culpable IAPs; the board bears a cost-benefit duty on D&amp;O coverage and on maintaining adequate fidelity bonds.</t>
+        </is>
+      </c>
+      <c r="F230" s="9" t="inlineStr">
+        <is>
+          <t>FDIC indemnification rule; §1818(n); OCC Director's Book</t>
+        </is>
+      </c>
+      <c r="G230" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 359; 12 U.S.C. 1818(n)</t>
+        </is>
+      </c>
+      <c r="H230" s="9" t="n"/>
+      <c r="I230" s="9" t="inlineStr">
+        <is>
+          <t>FDIC/OCC</t>
+        </is>
+      </c>
+      <c r="J230" s="9" t="inlineStr">
+        <is>
+          <t>BHC &amp; IDI</t>
+        </is>
+      </c>
+      <c r="K230" s="9" t="inlineStr">
+        <is>
+          <t>Full board / each director</t>
+        </is>
+      </c>
+      <c r="L230" s="9" t="inlineStr">
+        <is>
+          <t>Each director</t>
+        </is>
+      </c>
+      <c r="M230" s="9" t="inlineStr">
+        <is>
+          <t>Regulation / supervisory expectation</t>
+        </is>
+      </c>
+      <c r="N230" s="9" t="inlineStr">
+        <is>
+          <t>Prohibited-payment liability; personal loss exposure</t>
+        </is>
+      </c>
+      <c r="O230" s="9" t="inlineStr">
+        <is>
+          <t>Periodic / event-driven</t>
+        </is>
+      </c>
+      <c r="P230" s="10" t="inlineStr">
+        <is>
+          <t>n/a (individual)</t>
+        </is>
+      </c>
+      <c r="Q230" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="R230" s="11" t="inlineStr">
+        <is>
+          <t>Medium (Caffrey2-sourced; verify)</t>
+        </is>
+      </c>
+      <c r="S230" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="T230" s="9" t="inlineStr">
+        <is>
+          <t>Cross-cutting: single prudence objective enforced through three mechanisms with two culpability standards; tension between §1818(n) fee-shifting and Part 359's indemnification prohibition. Analytically distinct.</t>
         </is>
       </c>
     </row>
@@ -22837,7 +24895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -22881,7 +24939,7 @@
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
@@ -22896,7 +24954,7 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6">
@@ -22911,7 +24969,7 @@
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>197</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7">
@@ -22926,13 +24984,37 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>23</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Annual board actions (independent cross-check)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>v2.1: discrete, separately-documented board/committee actions required at least annually by a binding instrument (excludes proposed/withdrawn/rescinded and non-enforceable sound-practice guidance; no double-counting of a single vehicle binding both tiers; reflects the biennial Title I resolution cadence, 12 CFR 243.4(a)).</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>~70-75 (both tiers; ~20-25 incremental IDI)</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Note: Counts depend on the unit of analysis and counting granularity (e.g., the risk committee is one duty or seven sub-duties). Figures are a relative map, not an exact statutory tally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>v2.1 re-tally: headline counts now include the v2.1 additions — Narrow 55-&gt;68 (+13 in-force binding: credit-risk, fiduciary, director-eligibility), Medium 83-&gt;98 (+13 binding, +2 rule-backed expectations), Broad 197-&gt;214 (+13 binding, +4 expectations), duty-clusters 23-&gt;26 (+credit risk, fiduciary, director eligibility &amp; continuity). The 4 personal-liability rows are individual-director exposures, excluded from these board-duty totals. The action-count cross-check (~70-75) counts annual board ACTIONS, not duties.</t>
         </is>
       </c>
     </row>
@@ -22950,7 +25032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -23037,7 +25119,7 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>One enterprise framework approval with an IDI addendum.</t>
+          <t>One enterprise framework approval with an IDI addendum. v2.1: this expands the existing OCC Appendix D reliance accommodation, under which a covered bank may use the parent's framework in its entirety where the framework meets the minimum standards and parent/bank risk profiles are substantially the same — a partial mitigant already in law.</t>
         </is>
       </c>
     </row>
@@ -23048,7 +25130,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
@@ -23177,7 +25259,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Cross-reference manual to the rule; avoid restating.</t>
+          <t>Cross-reference manual to the rule; avoid restating. v2.1: resolve the two unreconciled pending rewrites (2024 proposals add a freestanding board-oversight standard + annual ratification; 2026 proposals permit approval by the board, an equivalent body, or senior management) before they compound the layering.</t>
         </is>
       </c>
     </row>
@@ -23258,7 +25340,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
@@ -23317,7 +25399,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>One enterprise info-security program approval; joint SEC/banking statement on cyber oversight.</t>
+          <t>One enterprise info-security program approval; joint SEC/banking statement on cyber oversight. v2.1: the 36-hour interagency incident-notification rule and the SEC cyber-disclosure regime impose non-aligned timelines on the same incident — harmonization here is selection of a single operational standard, not deletion.</t>
         </is>
       </c>
     </row>
@@ -23328,7 +25410,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
@@ -23608,7 +25690,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
@@ -23737,7 +25819,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Confirm the Heightened Standards do not re-impose the dropped board duty.</t>
+          <t>Confirm the Heightened Standards do not re-impose the dropped board duty. v2.1: SR 26-2 and OCC Bulletin 2026-13 (eff. Apr. 17, 2026) are expressly non-prescriptive and non-enforceable — neither should be cited as a binding board-approval mandate; any enforceable duty derives from 12 U.S.C. 1831p-1 / 12 CFR 30 App. D.</t>
         </is>
       </c>
     </row>
@@ -23808,6 +25890,146 @@
       <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Clarify the interaction for overlapping directors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Real Estate Lending Standards (parts 208/365/34); ACL policy statement; credit-risk-review guidance; Reg O; Reg W; Reg F</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Annual real-estate-lending policy approval, ACL oversight, and independent credit review stated in parallel across agency appendices and rules.</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Insider-credit (Reg O) and affiliate (Reg W) approvals protect the insured bank specifically.</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>One interagency real-estate-lending standard; fold ACL/credit-review into the risk-committee credit cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Fiduciary (trust) governance</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Unique / limited overlap</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>12 CFR part 9 (9.4/9.5/9.9/9.13/9.18)</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Board direction of fiduciary activities, written fiduciary policies, and a fiduciary audit committee (most material to BNY, State Street).</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Charter-specific trust duties distinct from enterprise risk governance.</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Permit the §36/Part 363 audit committee to satisfy the fiduciary-audit duty where composition overlaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Director eligibility &amp; continuity</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Candidate redundancy</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>12 U.S.C. 1831i; Reg Y 225.71-.73; OCC 5.51; 12 U.S.C. 1829; FDIA §8(e)/(g); FDI Act §7(a)(3)/(j)</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Parallel FRB/OCC change-in-director (914) notice regimes; statutory bars; report attestation.</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Statutory disqualification and Call Report attestation are unique, low-burden duties.</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Single interagency change-in-director notice procedure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Personal &amp; individual-director liability</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>n/a (individual; not a board action)</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>18 U.S.C. 1005; FDIA §8(e); 12 U.S.C. 1821(k)/5390(f)/5390(s); 12 CFR 359/380.7; §1818(n)</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Analytically distinct individual-director exposure (criminal, removal, receivership/OLA, indemnification) — amplifies cumulative burden.</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Runs to the individual director, not the board as a governance body; NOT counted as recurring board actions.</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Not a consolidation target; documented to show how personal liability compounds the cost of duplicative mandates.</t>
         </is>
       </c>
     </row>
@@ -23822,7 +26044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -24197,6 +26419,76 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Credit risk governance</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>CRD-01, CRD-02, CRD-03, CRD-04, CRD-05, CRD-06</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>CRD-02, CRD-03</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="18" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Fiduciary (trust) governance</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>FID-01, FID-03</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>FID-02</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>FID-02</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Director eligibility, attestation &amp; continuity</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>ELG-01, ELG-03, ELG-04</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>ELG-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -24208,7 +26500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -24650,6 +26942,50 @@
           <t>CON-03, CON-07</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Credit risk oversight (supervisory)</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>CRX-01, CRX-02</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>CRX-01, CRX-02</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="n"/>
+      <c r="F18" s="18" t="n"/>
+      <c r="G18" s="18" t="n"/>
+      <c r="H18" s="18" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Additional consumer &amp; compliance oversight</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>CCX-01, CCX-02</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>CCX-02</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26048,7 +28384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -26530,6 +28866,90 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Vertical (HC/IDI) rationalization via expanded reliance accommodation</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>FRB + OCC + FDIC</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>DFA §165; FDI Act §39; OCC Part 30 App. D</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Rulemaking (possibly statutory); expand App. D reliance accommodation</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Largest structural lever; removes the most pervasive overlap (parallel HC/IDI approve-oversee-report)</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Bank-board duty preserved via documented reliance where risk profiles are substantially the same; deposit-insurance interest retained</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Bank-level independent legal responsibility is statutory; reliance can be expanded but not eliminated</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Tiered feasibility principle (v2.1): harmonization is selection, not deletion</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>All agencies</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Sequence reforms by instrument: (1) guidance consolidation, (2) guidance retirement, (3) rule harmonization, (4) vertical HC/IDI rationalization, (5) statutory consolidation</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Varies by tier</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Orders the reforms above by legal feasibility; lowest cost at the guidance layer (2023 third-party guidance is the model)</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Each reform preserves the strictest substantive standard; only parallel documentation/examination footprint is removed</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Divergent standards (audit-committee independence; 36-hr vs SEC cyber timelines) require choosing a prevailing formulation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>